<commit_message>
Added HLD diagrams and started on the high level design decisions, comparing different architectures for our implementation
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/BRD-Review-Log-v0.1.xlsx
+++ b/docs/project-management/02_Business_Requirements/BRD-Review-Log-v0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="8_{A8AD7E28-50AD-41CA-B798-B213AEC76627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81CAF48C-042A-4EF6-BDF5-797DAC386BD3}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="8_{A8AD7E28-50AD-41CA-B798-B213AEC76627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{109B6CB4-69CC-437B-BD11-B22FFCC157A6}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{76AF004E-0D5E-43C6-8E8F-EE458AB65108}"/>
+    <workbookView xWindow="2145" yWindow="1770" windowWidth="21600" windowHeight="11295" firstSheet="5" activeTab="12" xr2:uid="{76AF004E-0D5E-43C6-8E8F-EE458AB65108}"/>
   </bookViews>
   <sheets>
     <sheet name="Workshop 2 Actions Log" sheetId="7" r:id="rId1"/>

</xml_diff>